<commit_message>
Update VNE project with ALIB implementation
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -447,7 +447,7 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
@@ -561,19 +561,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1411.812</v>
+        <v>877.0104</v>
       </c>
       <c r="C2" t="n">
-        <v>2879.6259</v>
+        <v>523.037</v>
       </c>
       <c r="D2" t="n">
-        <v>49.0276</v>
+        <v>167.6766</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>100</v>
@@ -582,34 +582,34 @@
         <v>840000</v>
       </c>
       <c r="I2" t="n">
-        <v>839672.0302028746</v>
+        <v>839793.2672516399</v>
       </c>
       <c r="J2" t="n">
-        <v>327.9697971254354</v>
+        <v>206.7327483601402</v>
       </c>
       <c r="K2" t="n">
-        <v>41.6862</v>
+        <v>41.8924</v>
       </c>
       <c r="L2" t="n">
-        <v>0.039</v>
+        <v>0.0246</v>
       </c>
       <c r="M2" t="n">
-        <v>0.7044</v>
+        <v>0.326</v>
       </c>
       <c r="N2" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O2" t="n">
-        <v>7.3333</v>
+        <v>7</v>
       </c>
       <c r="P2" t="n">
         <v>14</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.1923</v>
+        <v>4.6875</v>
       </c>
       <c r="R2" t="n">
-        <v>3899.5832</v>
+        <v>39360.8291</v>
       </c>
       <c r="S2" t="n">
         <v>840</v>
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -638,9 +638,9 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -703,32 +703,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PN1</t>
+          <t>PN2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>S125</t>
+          <t>S112</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1-&gt;78 | 2-&gt;21 | 3-&gt;52 | 4-&gt;43 | 5-&gt;6 | 6-&gt;47 | 7-&gt;71 | 8-&gt;45</t>
+          <t>1-&gt;43 | 2-&gt;37 | 3-&gt;6 | 4-&gt;71 | 5-&gt;35 | 6-&gt;9 | 7-&gt;4 | 8-&gt;45</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>7-8:71-&gt;1-&gt;45 | 5-8:6-&gt;71-&gt;1-&gt;45 | 2-4:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71-&gt;1-&gt;44-&gt;0-&gt;43 | 2-3:21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52 | 5-7:6-&gt;71 | 2-6:21-&gt;61-&gt;69-&gt;46-&gt;47 | 1-4:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71-&gt;1-&gt;44-&gt;0-&gt;43 | 2-5:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6 | 2-7:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71</t>
+          <t>3-4:6-&gt;71 | 1-3:43-&gt;0-&gt;44-&gt;1-&gt;71-&gt;6 | 6-8:9-&gt;8-&gt;75-&gt;29-&gt;7-&gt;30-&gt;45 | 5-8:35-&gt;40-&gt;41-&gt;43-&gt;0-&gt;44-&gt;1-&gt;45 | 1-4:43-&gt;0-&gt;44-&gt;1-&gt;71 | 7-8:4-&gt;10-&gt;55-&gt;13-&gt;75-&gt;29-&gt;7-&gt;30-&gt;45 | 2-6:37-&gt;60-&gt;11-&gt;55-&gt;10-&gt;9 | 1-8:43-&gt;0-&gt;44-&gt;1-&gt;45 | 4-8:71-&gt;1-&gt;45</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>-491.5223</v>
+        <v>195.9297</v>
       </c>
       <c r="H2" t="n">
         <v>501.5675</v>
       </c>
       <c r="I2" t="n">
-        <v>993.0898999999999</v>
+        <v>305.6378</v>
       </c>
     </row>
     <row r="3">
@@ -739,7 +739,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>vnet_8</t>
+          <t>vnet_3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -749,68 +749,27 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>S184</t>
+          <t>S95</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1-&gt;78 | 2-&gt;21 | 3-&gt;52 | 4-&gt;43 | 5-&gt;71 | 6-&gt;47 | 7-&gt;6 | 8-&gt;37</t>
+          <t>1-&gt;78 | 2-&gt;21 | 3-&gt;52 | 4-&gt;63 | 5-&gt;47 | 6-&gt;24</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2-6:21-&gt;61-&gt;69-&gt;46-&gt;47 | 4-7:43-&gt;0-&gt;44-&gt;1-&gt;71-&gt;6 | 2-7:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6 | 3-7:52-&gt;5-&gt;25-&gt;23-&gt;31-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6 | 3-4:52-&gt;60-&gt;11-&gt;55-&gt;13-&gt;75-&gt;29-&gt;7-&gt;30-&gt;45-&gt;1-&gt;44-&gt;0-&gt;43 | 1-5:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71 | 2-3:21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52 | 5-7:71-&gt;6 | 1-6:78-&gt;47 | 1-8:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52-&gt;60-&gt;37</t>
+          <t>2-6:21-&gt;18-&gt;31-&gt;24 | 1-5:78-&gt;47 | 2-3:21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52 | 2-4:21-&gt;18-&gt;16-&gt;63 | 2-5:21-&gt;61-&gt;69-&gt;46-&gt;47 | 3-6:52-&gt;5-&gt;27-&gt;26-&gt;28-&gt;24 | 1-3:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>-722.7095</v>
+        <v>158.0436</v>
       </c>
       <c r="H3" t="n">
-        <v>534.8016</v>
+        <v>375.4429</v>
       </c>
       <c r="I3" t="n">
-        <v>1257.5111</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>VNR3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>vnet_3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PN1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>S115</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1-&gt;37 | 2-&gt;35 | 3-&gt;4 | 4-&gt;9 | 5-&gt;27 | 6-&gt;8</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>4-6:9-&gt;8 | 3-5:4-&gt;65-&gt;5-&gt;27 | 1-6:37-&gt;60-&gt;11-&gt;55-&gt;13-&gt;75-&gt;8 | 2-6:35-&gt;40-&gt;41-&gt;43-&gt;0-&gt;44-&gt;1-&gt;45-&gt;30-&gt;7-&gt;29-&gt;75-&gt;8 | 3-6:4-&gt;10-&gt;9-&gt;8 | 1-4:37-&gt;60-&gt;11-&gt;55-&gt;10-&gt;9 | 1-5:37-&gt;60-&gt;52-&gt;5-&gt;27</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>-253.5821</v>
-      </c>
-      <c r="H4" t="n">
-        <v>375.4429</v>
-      </c>
-      <c r="I4" t="n">
-        <v>629.0249</v>
+        <v>217.3992</v>
       </c>
     </row>
   </sheetData>
@@ -824,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -832,8 +791,8 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -909,31 +868,31 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PN1</t>
+          <t>PN2</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>501.5675</v>
       </c>
       <c r="F2" t="n">
-        <v>993.0898999999999</v>
+        <v>305.6378</v>
       </c>
       <c r="G2" t="n">
-        <v>-491.5223</v>
+        <v>195.9297</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1-&gt;78 | 2-&gt;21 | 3-&gt;52 | 4-&gt;43 | 5-&gt;6 | 6-&gt;47 | 7-&gt;71 | 8-&gt;45</t>
+          <t>1-&gt;43 | 2-&gt;37 | 3-&gt;6 | 4-&gt;71 | 5-&gt;35 | 6-&gt;9 | 7-&gt;4 | 8-&gt;45</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7-8:71-&gt;1-&gt;45 | 5-8:6-&gt;71-&gt;1-&gt;45 | 2-4:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71-&gt;1-&gt;44-&gt;0-&gt;43 | 2-3:21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52 | 5-7:6-&gt;71 | 2-6:21-&gt;61-&gt;69-&gt;46-&gt;47 | 1-4:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71-&gt;1-&gt;44-&gt;0-&gt;43 | 2-5:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6 | 2-7:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71</t>
+          <t>3-4:6-&gt;71 | 1-3:43-&gt;0-&gt;44-&gt;1-&gt;71-&gt;6 | 6-8:9-&gt;8-&gt;75-&gt;29-&gt;7-&gt;30-&gt;45 | 5-8:35-&gt;40-&gt;41-&gt;43-&gt;0-&gt;44-&gt;1-&gt;45 | 1-4:43-&gt;0-&gt;44-&gt;1-&gt;71 | 7-8:4-&gt;10-&gt;55-&gt;13-&gt;75-&gt;29-&gt;7-&gt;30-&gt;45 | 2-6:37-&gt;60-&gt;11-&gt;55-&gt;10-&gt;9 | 1-8:43-&gt;0-&gt;44-&gt;1-&gt;45 | 4-8:71-&gt;1-&gt;45</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>S125</t>
+          <t>S112</t>
         </is>
       </c>
     </row>
@@ -945,7 +904,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>vnet_8</t>
+          <t>vnet_3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -959,73 +918,27 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>534.8016</v>
+        <v>375.4429</v>
       </c>
       <c r="F3" t="n">
-        <v>1257.5111</v>
+        <v>217.3992</v>
       </c>
       <c r="G3" t="n">
-        <v>-722.7095</v>
+        <v>158.0436</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1-&gt;78 | 2-&gt;21 | 3-&gt;52 | 4-&gt;43 | 5-&gt;71 | 6-&gt;47 | 7-&gt;6 | 8-&gt;37</t>
+          <t>1-&gt;78 | 2-&gt;21 | 3-&gt;52 | 4-&gt;63 | 5-&gt;47 | 6-&gt;24</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2-6:21-&gt;61-&gt;69-&gt;46-&gt;47 | 4-7:43-&gt;0-&gt;44-&gt;1-&gt;71-&gt;6 | 2-7:21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6 | 3-7:52-&gt;5-&gt;25-&gt;23-&gt;31-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6 | 3-4:52-&gt;60-&gt;11-&gt;55-&gt;13-&gt;75-&gt;29-&gt;7-&gt;30-&gt;45-&gt;1-&gt;44-&gt;0-&gt;43 | 1-5:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;22-&gt;20-&gt;48-&gt;54-&gt;6-&gt;71 | 2-3:21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52 | 5-7:71-&gt;6 | 1-6:78-&gt;47 | 1-8:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52-&gt;60-&gt;37</t>
+          <t>2-6:21-&gt;18-&gt;31-&gt;24 | 1-5:78-&gt;47 | 2-3:21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52 | 2-4:21-&gt;18-&gt;16-&gt;63 | 2-5:21-&gt;61-&gt;69-&gt;46-&gt;47 | 3-6:52-&gt;5-&gt;27-&gt;26-&gt;28-&gt;24 | 1-3:78-&gt;47-&gt;46-&gt;69-&gt;61-&gt;21-&gt;18-&gt;31-&gt;23-&gt;25-&gt;5-&gt;52</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>S184</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>VNR3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>vnet_3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>PN1</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>375.4429</v>
-      </c>
-      <c r="F4" t="n">
-        <v>629.0249</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-253.5821</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>1-&gt;37 | 2-&gt;35 | 3-&gt;4 | 4-&gt;9 | 5-&gt;27 | 6-&gt;8</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>4-6:9-&gt;8 | 3-5:4-&gt;65-&gt;5-&gt;27 | 1-6:37-&gt;60-&gt;11-&gt;55-&gt;13-&gt;75-&gt;8 | 2-6:35-&gt;40-&gt;41-&gt;43-&gt;0-&gt;44-&gt;1-&gt;45-&gt;30-&gt;7-&gt;29-&gt;75-&gt;8 | 3-6:4-&gt;10-&gt;9-&gt;8 | 1-4:37-&gt;60-&gt;11-&gt;55-&gt;10-&gt;9 | 1-5:37-&gt;60-&gt;52-&gt;5-&gt;27</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>S115</t>
+          <t>S95</t>
         </is>
       </c>
     </row>
@@ -1467,10 +1380,10 @@
         <v>1000</v>
       </c>
       <c r="E16" t="n">
-        <v>984.2734134702096</v>
+        <v>1000</v>
       </c>
       <c r="F16" t="n">
-        <v>15.72658652979044</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1623,10 +1536,10 @@
         <v>1000</v>
       </c>
       <c r="E22" t="n">
-        <v>985.9586697600397</v>
+        <v>1000</v>
       </c>
       <c r="F22" t="n">
-        <v>14.0413302399603</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1857,10 +1770,10 @@
         <v>1000</v>
       </c>
       <c r="E31" t="n">
-        <v>989.0546563696149</v>
+        <v>1000</v>
       </c>
       <c r="F31" t="n">
-        <v>10.94534363038508</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1909,10 +1822,10 @@
         <v>1000</v>
       </c>
       <c r="E33" t="n">
-        <v>986.7039443967994</v>
+        <v>1000</v>
       </c>
       <c r="F33" t="n">
-        <v>13.29605560320056</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1987,10 +1900,10 @@
         <v>1000</v>
       </c>
       <c r="E36" t="n">
-        <v>983.1782579514957</v>
+        <v>1000</v>
       </c>
       <c r="F36" t="n">
-        <v>16.82174204850435</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -2091,10 +2004,10 @@
         <v>1000</v>
       </c>
       <c r="E40" t="n">
-        <v>982.1220018487113</v>
+        <v>1000</v>
       </c>
       <c r="F40" t="n">
-        <v>17.87799815128869</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -2143,10 +2056,10 @@
         <v>1000</v>
       </c>
       <c r="E42" t="n">
-        <v>985.3262659722872</v>
+        <v>1000</v>
       </c>
       <c r="F42" t="n">
-        <v>14.67373402771284</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -2195,10 +2108,10 @@
         <v>1000</v>
       </c>
       <c r="E44" t="n">
-        <v>981.666992810135</v>
+        <v>1000</v>
       </c>
       <c r="F44" t="n">
-        <v>18.33300718986504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -2351,10 +2264,10 @@
         <v>1000</v>
       </c>
       <c r="E50" t="n">
-        <v>984.2052873939915</v>
+        <v>1000</v>
       </c>
       <c r="F50" t="n">
-        <v>15.79471260600849</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -2559,10 +2472,10 @@
         <v>1000</v>
       </c>
       <c r="E58" t="n">
-        <v>988.6397734785364</v>
+        <v>1000</v>
       </c>
       <c r="F58" t="n">
-        <v>11.36022652146357</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -2897,10 +2810,10 @@
         <v>1000</v>
       </c>
       <c r="E71" t="n">
-        <v>987.811860760849</v>
+        <v>1000</v>
       </c>
       <c r="F71" t="n">
-        <v>12.18813923915104</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -3079,10 +2992,10 @@
         <v>1000</v>
       </c>
       <c r="E78" t="n">
-        <v>988.6719609075482</v>
+        <v>1000</v>
       </c>
       <c r="F78" t="n">
-        <v>11.32803909245183</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -3131,10 +3044,10 @@
         <v>1000</v>
       </c>
       <c r="E80" t="n">
-        <v>982.2998407870296</v>
+        <v>1000</v>
       </c>
       <c r="F80" t="n">
-        <v>17.70015921297045</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -3261,10 +3174,10 @@
         <v>1000</v>
       </c>
       <c r="E85" t="n">
-        <v>983.3543257325509</v>
+        <v>1000</v>
       </c>
       <c r="F85" t="n">
-        <v>16.64567426744907</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3287,10 +3200,10 @@
         <v>1000</v>
       </c>
       <c r="E86" t="n">
-        <v>873.6247504750138</v>
+        <v>1000</v>
       </c>
       <c r="F86" t="n">
-        <v>126.3752495249862</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -3313,10 +3226,10 @@
         <v>1000</v>
       </c>
       <c r="E87" t="n">
-        <v>873.6247504750138</v>
+        <v>1000</v>
       </c>
       <c r="F87" t="n">
-        <v>126.3752495249862</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -3339,10 +3252,10 @@
         <v>1000</v>
       </c>
       <c r="E88" t="n">
-        <v>873.6247504750138</v>
+        <v>1000</v>
       </c>
       <c r="F88" t="n">
-        <v>126.3752495249862</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -3365,10 +3278,10 @@
         <v>1000</v>
       </c>
       <c r="E89" t="n">
-        <v>850.3334581859027</v>
+        <v>1000</v>
       </c>
       <c r="F89" t="n">
-        <v>149.6665418140973</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -3391,10 +3304,10 @@
         <v>1000</v>
       </c>
       <c r="E90" t="n">
-        <v>812.8629948346171</v>
+        <v>1000</v>
       </c>
       <c r="F90" t="n">
-        <v>187.1370051653829</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -3417,10 +3330,10 @@
         <v>1000</v>
       </c>
       <c r="E91" t="n">
-        <v>965.0815771709194</v>
+        <v>1000</v>
       </c>
       <c r="F91" t="n">
-        <v>34.91842282908055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -3443,10 +3356,10 @@
         <v>1000</v>
       </c>
       <c r="E92" t="n">
-        <v>968.2771614127111</v>
+        <v>1000</v>
       </c>
       <c r="F92" t="n">
-        <v>31.72283858728895</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -3469,10 +3382,10 @@
         <v>1000</v>
       </c>
       <c r="E93" t="n">
-        <v>933.3587385836305</v>
+        <v>1000</v>
       </c>
       <c r="F93" t="n">
-        <v>66.6412614163695</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -3495,10 +3408,10 @@
         <v>1000</v>
       </c>
       <c r="E94" t="n">
-        <v>922.5076073026971</v>
+        <v>1000</v>
       </c>
       <c r="F94" t="n">
-        <v>77.49239269730288</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -3521,10 +3434,10 @@
         <v>1000</v>
       </c>
       <c r="E95" t="n">
-        <v>922.5076073026971</v>
+        <v>1000</v>
       </c>
       <c r="F95" t="n">
-        <v>77.49239269730288</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -3625,10 +3538,10 @@
         <v>1000</v>
       </c>
       <c r="E99" t="n">
-        <v>954.230445889986</v>
+        <v>1000</v>
       </c>
       <c r="F99" t="n">
-        <v>45.76955411001404</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -3651,10 +3564,10 @@
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>954.230445889986</v>
+        <v>1000</v>
       </c>
       <c r="F100" t="n">
-        <v>45.76955411001404</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -3885,10 +3798,10 @@
         <v>1000</v>
       </c>
       <c r="E109" t="n">
-        <v>804.9686430021682</v>
+        <v>1000</v>
       </c>
       <c r="F109" t="n">
-        <v>195.0313569978318</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -3911,10 +3824,10 @@
         <v>1000</v>
       </c>
       <c r="E110" t="n">
-        <v>851.6028581491686</v>
+        <v>1000</v>
       </c>
       <c r="F110" t="n">
-        <v>148.3971418508314</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -3937,10 +3850,10 @@
         <v>1000</v>
       </c>
       <c r="E111" t="n">
-        <v>953.3657848529996</v>
+        <v>1000</v>
       </c>
       <c r="F111" t="n">
-        <v>46.63421514700042</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -4119,10 +4032,10 @@
         <v>1000</v>
       </c>
       <c r="E118" t="n">
-        <v>851.6028581491686</v>
+        <v>1000</v>
       </c>
       <c r="F118" t="n">
-        <v>148.3971418508314</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -4145,10 +4058,10 @@
         <v>1000</v>
       </c>
       <c r="E119" t="n">
-        <v>851.6028581491686</v>
+        <v>1000</v>
       </c>
       <c r="F119" t="n">
-        <v>148.3971418508314</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -4171,10 +4084,10 @@
         <v>1000</v>
       </c>
       <c r="E120" t="n">
-        <v>925.9311704012621</v>
+        <v>1000</v>
       </c>
       <c r="F120" t="n">
-        <v>74.06882959873792</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121">
@@ -4197,10 +4110,10 @@
         <v>1000</v>
       </c>
       <c r="E121" t="n">
-        <v>953.3657848529996</v>
+        <v>1000</v>
       </c>
       <c r="F121" t="n">
-        <v>46.63421514700042</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
@@ -4223,10 +4136,10 @@
         <v>1000</v>
       </c>
       <c r="E122" t="n">
-        <v>953.3657848529996</v>
+        <v>1000</v>
       </c>
       <c r="F122" t="n">
-        <v>46.63421514700042</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123">
@@ -4301,10 +4214,10 @@
         <v>1000</v>
       </c>
       <c r="E125" t="n">
-        <v>953.3657848529996</v>
+        <v>1000</v>
       </c>
       <c r="F125" t="n">
-        <v>46.63421514700042</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">
@@ -4379,10 +4292,10 @@
         <v>1000</v>
       </c>
       <c r="E128" t="n">
-        <v>920.4986008754503</v>
+        <v>1000</v>
       </c>
       <c r="F128" t="n">
-        <v>79.50139912454972</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -4405,10 +4318,10 @@
         <v>1000</v>
       </c>
       <c r="E129" t="n">
-        <v>955.5476069131497</v>
+        <v>1000</v>
       </c>
       <c r="F129" t="n">
-        <v>44.45239308685029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
@@ -4431,10 +4344,10 @@
         <v>1000</v>
       </c>
       <c r="E130" t="n">
-        <v>955.5476069131497</v>
+        <v>1000</v>
       </c>
       <c r="F130" t="n">
-        <v>44.45239308685029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -4483,10 +4396,10 @@
         <v>1000</v>
       </c>
       <c r="E132" t="n">
-        <v>955.5476069131497</v>
+        <v>1000</v>
       </c>
       <c r="F132" t="n">
-        <v>44.45239308685029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
@@ -4509,10 +4422,10 @@
         <v>1000</v>
       </c>
       <c r="E133" t="n">
-        <v>955.5476069131497</v>
+        <v>1000</v>
       </c>
       <c r="F133" t="n">
-        <v>44.45239308685029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -4639,10 +4552,10 @@
         <v>1000</v>
       </c>
       <c r="E138" t="n">
-        <v>955.5476069131497</v>
+        <v>1000</v>
       </c>
       <c r="F138" t="n">
-        <v>44.45239308685029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -4743,10 +4656,10 @@
         <v>1000</v>
       </c>
       <c r="E142" t="n">
-        <v>891.7481324285991</v>
+        <v>1000</v>
       </c>
       <c r="F142" t="n">
-        <v>108.2518675714009</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -4821,10 +4734,10 @@
         <v>1000</v>
       </c>
       <c r="E145" t="n">
-        <v>951.2580757495483</v>
+        <v>1000</v>
       </c>
       <c r="F145" t="n">
-        <v>48.74192425045169</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -4847,10 +4760,10 @@
         <v>1000</v>
       </c>
       <c r="E146" t="n">
-        <v>955.5476069131497</v>
+        <v>1000</v>
       </c>
       <c r="F146" t="n">
-        <v>44.45239308685029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -4899,10 +4812,10 @@
         <v>1000</v>
       </c>
       <c r="E148" t="n">
-        <v>955.5476069131497</v>
+        <v>1000</v>
       </c>
       <c r="F148" t="n">
-        <v>44.45239308685029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149">
@@ -4925,10 +4838,10 @@
         <v>1000</v>
       </c>
       <c r="E149" t="n">
-        <v>925.9311704012621</v>
+        <v>1000</v>
       </c>
       <c r="F149" t="n">
-        <v>74.06882959873792</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -4951,10 +4864,10 @@
         <v>1000</v>
       </c>
       <c r="E150" t="n">
-        <v>925.9311704012621</v>
+        <v>1000</v>
       </c>
       <c r="F150" t="n">
-        <v>74.06882959873792</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -4977,10 +4890,10 @@
         <v>1000</v>
       </c>
       <c r="E151" t="n">
-        <v>964.9408814491493</v>
+        <v>1000</v>
       </c>
       <c r="F151" t="n">
-        <v>35.05911855085071</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -5003,10 +4916,10 @@
         <v>1000</v>
       </c>
       <c r="E152" t="n">
-        <v>851.6028581491686</v>
+        <v>1000</v>
       </c>
       <c r="F152" t="n">
-        <v>148.3971418508314</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -5055,10 +4968,10 @@
         <v>1000</v>
       </c>
       <c r="E154" t="n">
-        <v>922.6063099789015</v>
+        <v>1000</v>
       </c>
       <c r="F154" t="n">
-        <v>77.39369002109845</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155">
@@ -5081,10 +4994,10 @@
         <v>1000</v>
       </c>
       <c r="E155" t="n">
-        <v>951.2580757495483</v>
+        <v>1000</v>
       </c>
       <c r="F155" t="n">
-        <v>48.74192425045169</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156">
@@ -5211,10 +5124,10 @@
         <v>1000</v>
       </c>
       <c r="E160" t="n">
-        <v>969.240525125902</v>
+        <v>1000</v>
       </c>
       <c r="F160" t="n">
-        <v>30.75947487409803</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -5237,10 +5150,10 @@
         <v>1000</v>
       </c>
       <c r="E161" t="n">
-        <v>851.6028581491686</v>
+        <v>1000</v>
       </c>
       <c r="F161" t="n">
-        <v>148.3971418508314</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162">
@@ -5367,10 +5280,10 @@
         <v>1000</v>
       </c>
       <c r="E166" t="n">
-        <v>790.047157220578</v>
+        <v>1000</v>
       </c>
       <c r="F166" t="n">
-        <v>209.952842779422</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167">
@@ -5393,10 +5306,10 @@
         <v>1000</v>
       </c>
       <c r="E167" t="n">
-        <v>925.9311704012621</v>
+        <v>1000</v>
       </c>
       <c r="F167" t="n">
-        <v>74.06882959873792</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -5575,10 +5488,10 @@
         <v>1000</v>
       </c>
       <c r="E174" t="n">
-        <v>909.7780528031358</v>
+        <v>1000</v>
       </c>
       <c r="F174" t="n">
-        <v>90.22194719686422</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -5679,10 +5592,10 @@
         <v>1000</v>
       </c>
       <c r="E178" t="n">
-        <v>915.4536268439844</v>
+        <v>1000</v>
       </c>
       <c r="F178" t="n">
-        <v>84.54637315601565</v>
+        <v>0</v>
       </c>
     </row>
     <row r="179">
@@ -6069,10 +5982,10 @@
         <v>1000</v>
       </c>
       <c r="E193" t="n">
-        <v>986.6729229514146</v>
+        <v>989.0546563696149</v>
       </c>
       <c r="F193" t="n">
-        <v>13.32707704858535</v>
+        <v>10.94534363038508</v>
       </c>
     </row>
     <row r="194">
@@ -6147,10 +6060,10 @@
         <v>1000</v>
       </c>
       <c r="E196" t="n">
-        <v>1000</v>
+        <v>982.2998407870296</v>
       </c>
       <c r="F196" t="n">
-        <v>0</v>
+        <v>17.70015921297045</v>
       </c>
     </row>
     <row r="197">
@@ -6459,10 +6372,10 @@
         <v>1000</v>
       </c>
       <c r="E208" t="n">
-        <v>1000</v>
+        <v>988.6397734785364</v>
       </c>
       <c r="F208" t="n">
-        <v>0</v>
+        <v>11.36022652146357</v>
       </c>
     </row>
     <row r="209">
@@ -6511,10 +6424,10 @@
         <v>1000</v>
       </c>
       <c r="E210" t="n">
-        <v>983.0527301735082</v>
+        <v>984.2734134702096</v>
       </c>
       <c r="F210" t="n">
-        <v>16.94726982649183</v>
+        <v>15.72658652979044</v>
       </c>
     </row>
     <row r="211">
@@ -6589,10 +6502,10 @@
         <v>1000</v>
       </c>
       <c r="E213" t="n">
-        <v>1000</v>
+        <v>987.811860760849</v>
       </c>
       <c r="F213" t="n">
-        <v>0</v>
+        <v>12.18813923915104</v>
       </c>
     </row>
     <row r="214">
@@ -6693,10 +6606,10 @@
         <v>1000</v>
       </c>
       <c r="E217" t="n">
-        <v>984.2787150068931</v>
+        <v>988.6719609075482</v>
       </c>
       <c r="F217" t="n">
-        <v>15.72128499310691</v>
+        <v>11.32803909245183</v>
       </c>
     </row>
     <row r="218">
@@ -6745,10 +6658,10 @@
         <v>1000</v>
       </c>
       <c r="E219" t="n">
-        <v>1000</v>
+        <v>985.3262659722872</v>
       </c>
       <c r="F219" t="n">
-        <v>0</v>
+        <v>14.67373402771284</v>
       </c>
     </row>
     <row r="220">
@@ -6797,10 +6710,10 @@
         <v>1000</v>
       </c>
       <c r="E221" t="n">
-        <v>982.6359764106754</v>
+        <v>985.9586697600397</v>
       </c>
       <c r="F221" t="n">
-        <v>17.36402358932457</v>
+        <v>14.0413302399603</v>
       </c>
     </row>
     <row r="222">
@@ -6953,10 +6866,10 @@
         <v>1000</v>
       </c>
       <c r="E227" t="n">
-        <v>986.9374145800117</v>
+        <v>983.1782579514957</v>
       </c>
       <c r="F227" t="n">
-        <v>13.0625854199883</v>
+        <v>16.82174204850435</v>
       </c>
     </row>
     <row r="228">
@@ -7161,10 +7074,10 @@
         <v>1000</v>
       </c>
       <c r="E235" t="n">
-        <v>984.8159739507099</v>
+        <v>984.2052873939915</v>
       </c>
       <c r="F235" t="n">
-        <v>15.18402604929008</v>
+        <v>15.79471260600849</v>
       </c>
     </row>
     <row r="236">
@@ -7265,10 +7178,10 @@
         <v>1000</v>
       </c>
       <c r="E239" t="n">
-        <v>1000</v>
+        <v>983.3543257325509</v>
       </c>
       <c r="F239" t="n">
-        <v>0</v>
+        <v>16.64567426744907</v>
       </c>
     </row>
     <row r="240">
@@ -7499,10 +7412,10 @@
         <v>1000</v>
       </c>
       <c r="E248" t="n">
-        <v>983.2478752676359</v>
+        <v>982.1220018487113</v>
       </c>
       <c r="F248" t="n">
-        <v>16.75212473236411</v>
+        <v>17.87799815128869</v>
       </c>
     </row>
     <row r="249">
@@ -7681,10 +7594,10 @@
         <v>1000</v>
       </c>
       <c r="E255" t="n">
-        <v>987.1213428938747</v>
+        <v>986.7039443967994</v>
       </c>
       <c r="F255" t="n">
-        <v>12.87865710612527</v>
+        <v>13.29605560320056</v>
       </c>
     </row>
     <row r="256">
@@ -7863,10 +7776,10 @@
         <v>1000</v>
       </c>
       <c r="E262" t="n">
-        <v>1000</v>
+        <v>981.666992810135</v>
       </c>
       <c r="F262" t="n">
-        <v>0</v>
+        <v>18.33300718986504</v>
       </c>
     </row>
     <row r="263">
@@ -7889,10 +7802,10 @@
         <v>1000</v>
       </c>
       <c r="E263" t="n">
-        <v>907.1072176980518</v>
+        <v>821.7672779259979</v>
       </c>
       <c r="F263" t="n">
-        <v>92.89278230194816</v>
+        <v>178.2327220740021</v>
       </c>
     </row>
     <row r="264">
@@ -7915,10 +7828,10 @@
         <v>1000</v>
       </c>
       <c r="E264" t="n">
-        <v>907.1072176980518</v>
+        <v>821.7672779259979</v>
       </c>
       <c r="F264" t="n">
-        <v>92.89278230194816</v>
+        <v>178.2327220740021</v>
       </c>
     </row>
     <row r="265">
@@ -7941,10 +7854,10 @@
         <v>1000</v>
       </c>
       <c r="E265" t="n">
-        <v>907.1072176980518</v>
+        <v>821.7672779259979</v>
       </c>
       <c r="F265" t="n">
-        <v>92.89278230194816</v>
+        <v>178.2327220740021</v>
       </c>
     </row>
     <row r="266">
@@ -7967,10 +7880,10 @@
         <v>1000</v>
       </c>
       <c r="E266" t="n">
-        <v>957.5501458123982</v>
+        <v>886.891499440304</v>
       </c>
       <c r="F266" t="n">
-        <v>42.44985418760177</v>
+        <v>113.108500559696</v>
       </c>
     </row>
     <row r="267">
@@ -7993,10 +7906,10 @@
         <v>1000</v>
       </c>
       <c r="E267" t="n">
-        <v>949.5570718856536</v>
+        <v>871.9700136587139</v>
       </c>
       <c r="F267" t="n">
-        <v>50.44292811434639</v>
+        <v>128.0299863412861</v>
       </c>
     </row>
     <row r="268">
@@ -8019,10 +7932,10 @@
         <v>1000</v>
       </c>
       <c r="E268" t="n">
-        <v>1000</v>
+        <v>960.9902889521128</v>
       </c>
       <c r="F268" t="n">
-        <v>0</v>
+        <v>39.00971104788721</v>
       </c>
     </row>
     <row r="269">
@@ -8045,10 +7958,10 @@
         <v>1000</v>
       </c>
       <c r="E269" t="n">
-        <v>1000</v>
+        <v>925.9311704012621</v>
       </c>
       <c r="F269" t="n">
-        <v>0</v>
+        <v>74.06882959873792</v>
       </c>
     </row>
     <row r="270">
@@ -8071,10 +7984,10 @@
         <v>1000</v>
       </c>
       <c r="E270" t="n">
-        <v>1000</v>
+        <v>964.9408814491493</v>
       </c>
       <c r="F270" t="n">
-        <v>0</v>
+        <v>35.05911855085071</v>
       </c>
     </row>
     <row r="271">
@@ -8097,10 +8010,10 @@
         <v>1000</v>
       </c>
       <c r="E271" t="n">
-        <v>957.5501458123982</v>
+        <v>964.9408814491493</v>
       </c>
       <c r="F271" t="n">
-        <v>42.44985418760177</v>
+        <v>35.05911855085071</v>
       </c>
     </row>
     <row r="272">
@@ -8123,10 +8036,10 @@
         <v>1000</v>
       </c>
       <c r="E272" t="n">
-        <v>957.5501458123982</v>
+        <v>964.9408814491493</v>
       </c>
       <c r="F272" t="n">
-        <v>42.44985418760177</v>
+        <v>35.05911855085071</v>
       </c>
     </row>
     <row r="273">
@@ -8227,10 +8140,10 @@
         <v>1000</v>
       </c>
       <c r="E276" t="n">
-        <v>957.5501458123982</v>
+        <v>960.9902889521128</v>
       </c>
       <c r="F276" t="n">
-        <v>42.44985418760177</v>
+        <v>39.00971104788721</v>
       </c>
     </row>
     <row r="277">
@@ -8253,10 +8166,10 @@
         <v>1000</v>
       </c>
       <c r="E277" t="n">
-        <v>957.5501458123982</v>
+        <v>960.9902889521128</v>
       </c>
       <c r="F277" t="n">
-        <v>42.44985418760177</v>
+        <v>39.00971104788721</v>
       </c>
     </row>
     <row r="278">
@@ -8383,10 +8296,10 @@
         <v>1000</v>
       </c>
       <c r="E282" t="n">
-        <v>1000</v>
+        <v>955.5476069131497</v>
       </c>
       <c r="F282" t="n">
-        <v>0</v>
+        <v>44.45239308685029</v>
       </c>
     </row>
     <row r="283">
@@ -8409,10 +8322,10 @@
         <v>1000</v>
       </c>
       <c r="E283" t="n">
-        <v>1000</v>
+        <v>955.5476069131497</v>
       </c>
       <c r="F283" t="n">
-        <v>0</v>
+        <v>44.45239308685029</v>
       </c>
     </row>
     <row r="284">
@@ -8487,10 +8400,10 @@
         <v>1000</v>
       </c>
       <c r="E286" t="n">
-        <v>844.7008589855413</v>
+        <v>829.3906276021027</v>
       </c>
       <c r="F286" t="n">
-        <v>155.2991410144587</v>
+        <v>170.6093723978973</v>
       </c>
     </row>
     <row r="287">
@@ -8513,10 +8426,10 @@
         <v>1000</v>
       </c>
       <c r="E287" t="n">
-        <v>867.5623695642515</v>
+        <v>1000</v>
       </c>
       <c r="F287" t="n">
-        <v>132.4376304357485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="288">
@@ -8539,10 +8452,10 @@
         <v>1000</v>
       </c>
       <c r="E288" t="n">
-        <v>889.3596812240429</v>
+        <v>873.8430206889529</v>
       </c>
       <c r="F288" t="n">
-        <v>110.6403187759571</v>
+        <v>126.1569793110471</v>
       </c>
     </row>
     <row r="289">
@@ -8721,10 +8634,10 @@
         <v>1000</v>
       </c>
       <c r="E295" t="n">
-        <v>867.5623695642515</v>
+        <v>1000</v>
       </c>
       <c r="F295" t="n">
-        <v>132.4376304357485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="296">
@@ -8747,10 +8660,10 @@
         <v>1000</v>
       </c>
       <c r="E296" t="n">
-        <v>867.5623695642515</v>
+        <v>1000</v>
       </c>
       <c r="F296" t="n">
-        <v>132.4376304357485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="297">
@@ -8773,10 +8686,10 @@
         <v>1000</v>
       </c>
       <c r="E297" t="n">
-        <v>876.4348010889347</v>
+        <v>934.3221022968214</v>
       </c>
       <c r="F297" t="n">
-        <v>123.5651989110653</v>
+        <v>65.67789770317859</v>
       </c>
     </row>
     <row r="298">
@@ -8799,10 +8712,10 @@
         <v>1000</v>
       </c>
       <c r="E298" t="n">
-        <v>889.3596812240429</v>
+        <v>923.4709710158879</v>
       </c>
       <c r="F298" t="n">
-        <v>110.6403187759571</v>
+        <v>76.52902898411207</v>
       </c>
     </row>
     <row r="299">
@@ -8825,10 +8738,10 @@
         <v>1000</v>
       </c>
       <c r="E299" t="n">
-        <v>889.3596812240429</v>
+        <v>923.4709710158879</v>
       </c>
       <c r="F299" t="n">
-        <v>110.6403187759571</v>
+        <v>76.52902898411207</v>
       </c>
     </row>
     <row r="300">
@@ -8851,10 +8764,10 @@
         <v>1000</v>
       </c>
       <c r="E300" t="n">
-        <v>1000</v>
+        <v>968.2771614127111</v>
       </c>
       <c r="F300" t="n">
-        <v>0</v>
+        <v>31.72283858728895</v>
       </c>
     </row>
     <row r="301">
@@ -8877,10 +8790,10 @@
         <v>1000</v>
       </c>
       <c r="E301" t="n">
-        <v>1000</v>
+        <v>950.3720496730649</v>
       </c>
       <c r="F301" t="n">
-        <v>0</v>
+        <v>49.62795032693509</v>
       </c>
     </row>
     <row r="302">
@@ -8903,10 +8816,10 @@
         <v>1000</v>
       </c>
       <c r="E302" t="n">
-        <v>889.3596812240429</v>
+        <v>923.4709710158879</v>
       </c>
       <c r="F302" t="n">
-        <v>110.6403187759571</v>
+        <v>76.52902898411207</v>
       </c>
     </row>
     <row r="303">
@@ -8929,10 +8842,10 @@
         <v>1000</v>
       </c>
       <c r="E303" t="n">
-        <v>1000</v>
+        <v>968.2771614127111</v>
       </c>
       <c r="F303" t="n">
-        <v>0</v>
+        <v>31.72283858728895</v>
       </c>
     </row>
     <row r="304">
@@ -8955,10 +8868,10 @@
         <v>1000</v>
       </c>
       <c r="E304" t="n">
-        <v>1000</v>
+        <v>968.2771614127111</v>
       </c>
       <c r="F304" t="n">
-        <v>0</v>
+        <v>31.72283858728895</v>
       </c>
     </row>
     <row r="305">
@@ -8981,10 +8894,10 @@
         <v>1000</v>
       </c>
       <c r="E305" t="n">
-        <v>1000</v>
+        <v>968.2771614127111</v>
       </c>
       <c r="F305" t="n">
-        <v>0</v>
+        <v>31.72283858728895</v>
       </c>
     </row>
     <row r="306">
@@ -9007,10 +8920,10 @@
         <v>1000</v>
       </c>
       <c r="E306" t="n">
-        <v>957.5501458123982</v>
+        <v>914.1265510648277</v>
       </c>
       <c r="F306" t="n">
-        <v>42.44985418760177</v>
+        <v>85.87344893517229</v>
       </c>
     </row>
     <row r="307">
@@ -9033,10 +8946,10 @@
         <v>1000</v>
       </c>
       <c r="E307" t="n">
-        <v>957.5501458123982</v>
+        <v>914.1265510648277</v>
       </c>
       <c r="F307" t="n">
-        <v>42.44985418760177</v>
+        <v>85.87344893517229</v>
       </c>
     </row>
     <row r="308">
@@ -9085,10 +8998,10 @@
         <v>1000</v>
       </c>
       <c r="E309" t="n">
-        <v>957.5501458123982</v>
+        <v>914.1265510648277</v>
       </c>
       <c r="F309" t="n">
-        <v>42.44985418760177</v>
+        <v>85.87344893517229</v>
       </c>
     </row>
     <row r="310">
@@ -9111,10 +9024,10 @@
         <v>1000</v>
       </c>
       <c r="E310" t="n">
-        <v>957.5501458123982</v>
+        <v>914.1265510648277</v>
       </c>
       <c r="F310" t="n">
-        <v>42.44985418760177</v>
+        <v>85.87344893517229</v>
       </c>
     </row>
     <row r="311">
@@ -9241,10 +9154,10 @@
         <v>1000</v>
       </c>
       <c r="E315" t="n">
-        <v>1000</v>
+        <v>953.3657848529996</v>
       </c>
       <c r="F315" t="n">
-        <v>0</v>
+        <v>46.63421514700042</v>
       </c>
     </row>
     <row r="316">
@@ -9345,10 +9258,10 @@
         <v>1000</v>
       </c>
       <c r="E319" t="n">
-        <v>968.9270437165405</v>
+        <v>964.9408814491493</v>
       </c>
       <c r="F319" t="n">
-        <v>31.07295628345946</v>
+        <v>35.05911855085071</v>
       </c>
     </row>
     <row r="320">
@@ -9449,10 +9362,10 @@
         <v>1000</v>
       </c>
       <c r="E323" t="n">
-        <v>1000</v>
+        <v>953.3657848529996</v>
       </c>
       <c r="F323" t="n">
-        <v>0</v>
+        <v>46.63421514700042</v>
       </c>
     </row>
     <row r="324">
@@ -9501,10 +9414,10 @@
         <v>1000</v>
       </c>
       <c r="E325" t="n">
-        <v>1000</v>
+        <v>953.3657848529996</v>
       </c>
       <c r="F325" t="n">
-        <v>0</v>
+        <v>46.63421514700042</v>
       </c>
     </row>
     <row r="326">
@@ -9527,10 +9440,10 @@
         <v>1000</v>
       </c>
       <c r="E326" t="n">
-        <v>876.4348010889347</v>
+        <v>934.3221022968214</v>
       </c>
       <c r="F326" t="n">
-        <v>123.5651989110653</v>
+        <v>65.67789770317859</v>
       </c>
     </row>
     <row r="327">
@@ -9553,10 +9466,10 @@
         <v>1000</v>
       </c>
       <c r="E327" t="n">
-        <v>876.4348010889347</v>
+        <v>934.3221022968214</v>
       </c>
       <c r="F327" t="n">
-        <v>123.5651989110653</v>
+        <v>65.67789770317859</v>
       </c>
     </row>
     <row r="328">
@@ -9579,10 +9492,10 @@
         <v>1000</v>
       </c>
       <c r="E328" t="n">
-        <v>895.7575272428282</v>
+        <v>920.4986008754503</v>
       </c>
       <c r="F328" t="n">
-        <v>104.2424727571718</v>
+        <v>79.50139912454972</v>
       </c>
     </row>
     <row r="329">
@@ -9605,10 +9518,10 @@
         <v>1000</v>
       </c>
       <c r="E329" t="n">
-        <v>867.5623695642515</v>
+        <v>1000</v>
       </c>
       <c r="F329" t="n">
-        <v>132.4376304357485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330">
@@ -9657,10 +9570,10 @@
         <v>1000</v>
       </c>
       <c r="E331" t="n">
-        <v>889.3596812240429</v>
+        <v>891.7481324285991</v>
       </c>
       <c r="F331" t="n">
-        <v>110.6403187759571</v>
+        <v>108.2518675714009</v>
       </c>
     </row>
     <row r="332">
@@ -9813,10 +9726,10 @@
         <v>1000</v>
       </c>
       <c r="E337" t="n">
-        <v>926.4771895289388</v>
+        <v>1000</v>
       </c>
       <c r="F337" t="n">
-        <v>73.52281047106123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="338">
@@ -9839,10 +9752,10 @@
         <v>1000</v>
       </c>
       <c r="E338" t="n">
-        <v>867.5623695642515</v>
+        <v>1000</v>
       </c>
       <c r="F338" t="n">
-        <v>132.4376304357485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="339">
@@ -9969,10 +9882,10 @@
         <v>1000</v>
       </c>
       <c r="E343" t="n">
-        <v>874.1676939289115</v>
+        <v>894.785851272753</v>
       </c>
       <c r="F343" t="n">
-        <v>125.8323060710885</v>
+        <v>105.214148727247</v>
       </c>
     </row>
     <row r="344">
@@ -9995,10 +9908,10 @@
         <v>1000</v>
       </c>
       <c r="E344" t="n">
-        <v>876.4348010889347</v>
+        <v>934.3221022968214</v>
       </c>
       <c r="F344" t="n">
-        <v>123.5651989110653</v>
+        <v>65.67789770317859</v>
       </c>
     </row>
     <row r="345">
@@ -10177,10 +10090,10 @@
         <v>1000</v>
       </c>
       <c r="E351" t="n">
-        <v>1000</v>
+        <v>953.1362621127148</v>
       </c>
       <c r="F351" t="n">
-        <v>0</v>
+        <v>46.8637378872852</v>
       </c>
     </row>
     <row r="352">
@@ -10281,10 +10194,10 @@
         <v>1000</v>
       </c>
       <c r="E355" t="n">
-        <v>1000</v>
+        <v>953.1362621127148</v>
       </c>
       <c r="F355" t="n">
-        <v>0</v>
+        <v>46.8637378872852</v>
       </c>
     </row>
     <row r="356">
@@ -47122,7 +47035,7 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="31" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -47169,10 +47082,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9</v>
+        <v>0.651071</v>
       </c>
       <c r="D2" t="n">
-        <v>0.394531</v>
+        <v>0.128124</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -47180,7 +47093,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-2879.6259</v>
+        <v>-523.037</v>
       </c>
     </row>
   </sheetData>
@@ -47194,7 +47107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -47219,7 +47132,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'Iteration': 1, 'VNR': 'vnet_5', 'Network': 'PN1', 'Decision': 'UPDATED', 'Utility': -491.5223, 'Cost': 993.0899}</t>
+          <t>{'Iteration': 1, 'VNR': 'vnet_5', 'Network': 'PN1', 'Decision': 'UPDATED', 'Utility': 7.4996, 'Cost': 494.0679}</t>
         </is>
       </c>
     </row>
@@ -47229,7 +47142,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'Iteration': 1, 'VNR': 'vnet_8', 'Network': 'PN2', 'Decision': 'UPDATED', 'Utility': -722.7095, 'Cost': 1257.5111}</t>
+          <t>{'Iteration': 1, 'VNR': 'vnet_3', 'Network': 'PN2', 'Decision': 'UPDATED', 'Utility': 121.3581, 'Cost': 254.0847}</t>
         </is>
       </c>
     </row>
@@ -47239,7 +47152,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{'Iteration': 1, 'VNR': 'vnet_3', 'Network': 'PN1', 'Decision': 'UPDATED', 'Utility': -253.5821, 'Cost': 629.0249}</t>
+          <t>{'Iteration': 2, 'VNR': 'vnet_5', 'Network': 'PN2', 'Decision': 'UPDATED', 'Utility': 103.1724, 'Cost': 398.3951}</t>
         </is>
       </c>
     </row>
@@ -47249,7 +47162,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{'Iteration': 2, 'VNR': 'vnet_5', 'Network': 'PN1', 'Decision': 'NO_CHANGE', 'Utility': -491.5223}</t>
+          <t>{'Iteration': 2, 'VNR': 'vnet_3', 'Network': 'PN2', 'Decision': 'UPDATED', 'Utility': 140.9574, 'Cost': 234.4855}</t>
         </is>
       </c>
     </row>
@@ -47259,7 +47172,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{'Iteration': 2, 'VNR': 'vnet_8', 'Network': 'PN2', 'Decision': 'NO_CHANGE', 'Utility': -722.7095}</t>
+          <t>{'Iteration': 3, 'VNR': 'vnet_5', 'Network': 'PN2', 'Decision': 'UPDATED', 'Utility': 138.8286, 'Cost': 362.7389}</t>
         </is>
       </c>
     </row>
@@ -47269,7 +47182,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{'Iteration': 2, 'VNR': 'vnet_3', 'Network': 'PN1', 'Decision': 'NO_CHANGE', 'Utility': -253.5821}</t>
+          <t>{'Iteration': 3, 'VNR': 'vnet_3', 'Network': 'PN2', 'Decision': 'UPDATED', 'Utility': 158.0436, 'Cost': 217.3992}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>{'Iteration': 4, 'VNR': 'vnet_5', 'Network': 'PN2', 'Decision': 'UPDATED', 'Utility': 195.9297, 'Cost': 305.6378}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{'Iteration': 4, 'VNR': 'vnet_3', 'Network': 'PN2', 'Decision': 'NO_CHANGE', 'Utility': 158.0436}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>{'Iteration': 5, 'VNR': 'vnet_5', 'Network': 'PN2', 'Decision': 'NO_CHANGE', 'Utility': 195.9297}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>{'Iteration': 5, 'VNR': 'vnet_3', 'Network': 'PN2', 'Decision': 'NO_CHANGE', 'Utility': 158.0436}</t>
         </is>
       </c>
     </row>

</xml_diff>